<commit_message>
feat: add period-scoped multimedia chronicles and tactical loadouts
</commit_message>
<xml_diff>
--- a/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Galaxy_Production.xlsx
+++ b/docs/universe/outputs/relay-chronicles-20261022/Mass_Effect_Galaxy_Production.xlsx
@@ -2,34 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6bf74bc4b6e84ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="Rc1fb6a9e859649eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="R8c3eb507bd054789"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="R71327b22078b45a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="Rc4b70f4a9de64d6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="Rf50c537654de48ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="R6b283ef6473f4de9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="Rcc6ffdbc42ab4fdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="Raa5716ae928f435d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="R97a29a65a0624e3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="R02f5128e1e3541e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="R431a334ce6194bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="Rda77e14ec20242c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="Rde214a584c6b4be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="R6752792bcd604482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="R99ce3f218bcd4c6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="R3ee63873543f4577"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="R6c943191c43b44bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="R7241c07809d14949"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="R2e1a326aea494627"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="R53a3e51abb4f4cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="R7a51d589565e4318"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="R25856e42362940df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="R0f82bbb2f27d4715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="R845ed21b3f0049d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="R2cc8eda18e1f4017"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="R0621a6042eb846f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R4715612e11534838"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0fb0a4a5a5ca4ec2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personnages" sheetId="2" r:id="R5113a7bb2cdf409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNJ" sheetId="3" r:id="R70bae102b1854b7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especes_factions" sheetId="4" r:id="R7ecdf795f67c4157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mondes" sheetId="5" r:id="R0aaaf6dc91b94058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zones" sheetId="6" r:id="R5994327c80ca4caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liaisons" sheetId="7" r:id="Rc97ebb8921134f59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decors" sheetId="8" r:id="R58845d09dfba4777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="9" r:id="R29f4b939263c43d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ennemis_boss" sheetId="10" r:id="Rf0b0c12b686347a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missions" sheetId="11" r:id="R30cbd3a4f26942a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secondaires_DLC" sheetId="12" r:id="Rffbfb02215024dee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choix_relations" sheetId="13" r:id="R484cd508ee3e4386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dialogues" sheetId="14" r:id="R65121cf36d8f4575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cinematiques" sheetId="15" r:id="R4e44cf14fb3c4887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armes" sheetId="16" r:id="R84b9443bc7f24736"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armures_equipement" sheetId="17" r:id="Rb6547729c9f645a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pouvoirs" sheetId="18" r:id="Rf8a5c1665c4a4a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_allies" sheetId="19" r:id="R8915b8edc51649c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movesets_ennemis" sheetId="20" r:id="R58f02fb46b4d47cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="21" r:id="Recd17ccada6e4534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprites" sheetId="22" r:id="Rae8ad2a9b2d14063"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VFX" sheetId="23" r:id="Rd6076f23be084487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="24" r:id="R83477b77f6db4b9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI_systemes" sheetId="25" r:id="Rc665eb1889ab4e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="26" r:id="R6dc247f76ed64bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuite" sheetId="27" r:id="R99c1ee1e58c94809"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="28" r:id="R5a534ebc94234915"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2285,11 +2285,11 @@
       </x:c>
       <x:c r="C10" s="39" t="n">
         <x:f>COUNTIFS('Personnages'!$C$7:$C$8,"Défini")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="39" t="n">
         <x:f>COUNTIFS('Personnages'!$C$7:$C$8,"Prototype")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="39" t="n">
         <x:f>COUNTIFS('Personnages'!$C$7:$C$8,"Intégré")</x:f>
@@ -3678,11 +3678,11 @@
       </x:c>
       <x:c r="C37" s="41" t="n">
         <x:f>SUM(C10:C35)</x:f>
-        <x:v>103</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D37" s="41" t="n">
         <x:f>SUM(D10:D35)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E37" s="41" t="n">
         <x:f>SUM(E10:E35)</x:f>
@@ -4226,7 +4226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0c2557068e549fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc571e334ef964e2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4772,7 +4772,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71e71f25f3494147"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3d4e8460db94439"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5131,7 +5131,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re944c5a14b6f48bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb46aa061918a414e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5492,7 +5492,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R982fb354f1534dba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77a758fbed9c454b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5851,7 +5851,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d2a65ec3da46b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c1d1c7f63af437d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6210,7 +6210,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc785e9a1a82a4f3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4cd34042e22448f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6534,7 +6534,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4191a949b5a460d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2ac74b8747d43b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6858,7 +6858,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7601ce49fa7a45d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903dcd126bb84832"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7229,7 +7229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0886e4c5714564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref955c5c6cb64805"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7663,7 +7663,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1c6ad09fc3b4ff8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5ad1d9f3d314997"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7690,7 +7690,7 @@
     <x:col min="16" max="16" width="45" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="69" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="73" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="247" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">
@@ -7861,7 +7861,7 @@
         <x:v>Notes et limites</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="44" customHeight="1">
+    <x:row r="7" ht="68" customHeight="1">
       <x:c r="A7" s="18" t="str">
         <x:v>GAL-CHR-JACOB</x:v>
       </x:c>
@@ -7869,7 +7869,7 @@
         <x:v>Jacob Taylor</x:v>
       </x:c>
       <x:c r="C7" s="15" t="str">
-        <x:v>Défini</x:v>
+        <x:v>Prototype</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>Établi</x:v>
@@ -7891,7 +7891,9 @@
       </x:c>
       <x:c r="J7" s="9" t="str"/>
       <x:c r="K7" s="9" t="str"/>
-      <x:c r="L7" s="9" t="str"/>
+      <x:c r="L7" s="9" t="str">
+        <x:v>Prototype Chroniques : src/universe-actors.js, src/chronicles.js. Identifiant runtime GAL-CHR-JACOB ; contexte d’œuvre/segment et sélection de scène obligatoires.</x:v>
+      </x:c>
       <x:c r="M7" s="9" t="str"/>
       <x:c r="N7" s="9" t="str">
         <x:v>La fiche distingue identité de référence et rôle proposé.</x:v>
@@ -7907,7 +7909,7 @@
         <x:v>https://masseffect.fandom.com/wiki/Mass_Effect_Galaxy</x:v>
       </x:c>
       <x:c r="S7" s="20" t="str">
-        <x:v>Costume exact à contrôler sur les images originales avant validation 1:1.</x:v>
+        <x:v>Costume exact à contrôler sur les images originales avant validation 1:1. Prototype partiel disponible dans les Chroniques indépendantes : profil ATB sans portrait, sprite ou moveset complet ; pouvoirs non implémentés signalés. Aucun transfert vers ME1 ni validation 1:1.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="44" customHeight="1">
@@ -7991,7 +7993,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb94b846eb71485b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d1cac69d7934623"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8417,7 +8419,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a664445e0f54fb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dce37c5ddfc4565"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8733,7 +8735,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R621404a63e4746ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20bae8a47a1f4221"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9599,7 +9601,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R426ead60212f447e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde85ba6141214abc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9915,7 +9917,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf897973cf2244cd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaee45370b164efe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10268,7 +10270,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b0f8cf84b244b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R411556d03d464dc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10713,7 +10715,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18ad9aae0eee4985"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb93e59ae9b1e4a74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11148,7 +11150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1011b536b3fb4d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c8750dbed11451c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11507,7 +11509,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77ad306eb7694052"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51fafea38ff649ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11619,12 +11621,12 @@
       <x:c r="E9" s="2"/>
       <x:c r="F9" s="2"/>
     </x:row>
-    <x:row r="10" ht="40" customHeight="1">
+    <x:row r="10" ht="68" customHeight="1">
       <x:c r="A10" s="7" t="str">
         <x:v>Projet</x:v>
       </x:c>
       <x:c r="B10" s="7" t="str">
-        <x:v>Transformer les arènes mobiles et la narration dessinée en module ATB de poche, avec décors 3D.</x:v>
+        <x:v>Transformer les arènes mobiles et la narration dessinée en module ATB de poche, avec décors 3D. Prototype partiel : 1 profils sélectionnables et 0 équipements en Chroniques ; le reste demeure documentaire.</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -11643,7 +11645,7 @@
       <x:c r="E11" s="2"/>
       <x:c r="F11" s="2"/>
     </x:row>
-    <x:row r="12" ht="40" customHeight="1">
+    <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="7" t="str">
         <x:v>Date de référence</x:v>
       </x:c>
@@ -12093,10 +12095,16 @@
       <x:c r="E43" s="2"/>
       <x:c r="F43" s="2"/>
     </x:row>
-    <x:row r="44" ht="22" customHeight="1">
-      <x:c r="A44" s="2"/>
-      <x:c r="B44" s="2"/>
-      <x:c r="C44" s="2"/>
+    <x:row r="44" ht="96" customHeight="1">
+      <x:c r="A44" s="6" t="str">
+        <x:v>Prototype Chroniques indépendant</x:v>
+      </x:c>
+      <x:c r="B44" s="6" t="str">
+        <x:v>1 personnages sélectionnables, 0 équipements utilisables sous restrictions d’œuvre, segment, scène et porteur ; preuves dans implementationPaths et evidence des seules lignes Prototype.</x:v>
+      </x:c>
+      <x:c r="C44" s="6" t="str">
+        <x:v>Campagne complète, dialogues, acquisition canonique, sprites, costumes, animations et statistiques originales à réaliser ou vérifier. Les ateliers sont des essais de préparation ATB, sans progression canonique ni transfert ME1.</x:v>
+      </x:c>
       <x:c r="D44" s="2"/>
       <x:c r="E44" s="2"/>
       <x:c r="F44" s="2"/>
@@ -12652,6 +12660,14 @@
       <x:c r="D113" s="2"/>
       <x:c r="E113" s="2"/>
       <x:c r="F113" s="2"/>
+    </x:row>
+    <x:row r="114" ht="22" customHeight="1">
+      <x:c r="A114" s="2"/>
+      <x:c r="B114" s="2"/>
+      <x:c r="C114" s="2"/>
+      <x:c r="D114" s="2"/>
+      <x:c r="E114" s="2"/>
+      <x:c r="F114" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13165,7 +13181,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38794e8b42b3488d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c713990336a4e2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13534,7 +13550,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68ee821f95aa4183"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f631e239ff2466e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14046,7 +14062,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R256f86640cfc4142"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R533fb181f3cd4128"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14570,7 +14586,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re04ddb9102394d7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20d84c059a464f8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14895,7 +14911,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8762300bf1d44b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a416c9ed594484a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15431,7 +15447,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdead282dc02843fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R788f8d474d554918"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15790,7 +15806,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5536f3777614c3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05f4c9d781bd4cc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>